<commit_message>
tools: dedup HumanLabel + preserve (Overflow)/(abs)/(rel)/section-prefix disambiguation
</commit_message>
<xml_diff>
--- a/dev/humanlabel-review.xlsx
+++ b/dev/humanlabel-review.xlsx
@@ -578,7 +578,7 @@
       <c r="A3" t="inlineStr"/>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Lights Toggle</t>
+          <t>Cabin Lights Toggle</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -619,7 +619,7 @@
       <c r="A4" t="inlineStr"/>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Lights Toggle</t>
+          <t>Running Lights Toggle</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1203,7 +1203,7 @@
       <c r="A16" t="inlineStr"/>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Fire Disintegrate Toggle</t>
+          <t>Fire Disintegrate</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1252,7 +1252,7 @@
       <c r="A17" t="inlineStr"/>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Fire Focused Salvage Beam Toggle</t>
+          <t>Salvage Fire Focused Toggle</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1888,7 +1888,7 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Door Lock Cycle</t>
+          <t>Pinned Target Forward</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -2141,7 +2141,7 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Next Weapon Preset</t>
+          <t>Next Weapon Preset (Overflow)</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -2769,7 +2769,7 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Chat Window Toggle</t>
+          <t>Chat Window Focus</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -3014,7 +3014,7 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Chat Window Toggle</t>
+          <t>Chat Window</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>Speed Limiter Inc. Step</t>
+          <t>Default Movement Speed Inc.</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -3512,7 +3512,7 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>Look Behind</t>
+          <t>Look (Yaw)</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -3798,7 +3798,7 @@
       <c r="A67" t="inlineStr"/>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>Previous Remote Turret*</t>
+          <t>Prev. Item</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -4035,7 +4035,7 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>Flashlight Toggle</t>
+          <t>Flashlight</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -4207,7 +4207,7 @@
       <c r="A76" t="inlineStr"/>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>Turret Zoom</t>
+          <t>Zoom In</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -4256,7 +4256,7 @@
       <c r="A77" t="inlineStr"/>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>Turret Zoom</t>
+          <t>Zoom Out</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -4403,7 +4403,7 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>Exit Remote Turret</t>
+          <t>Exit</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -4603,7 +4603,7 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>Focus Right Tool</t>
+          <t>MFD Right</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -4750,7 +4750,7 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>Turret Zoom</t>
+          <t>Interaction Mode Zoom In</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -4803,7 +4803,7 @@
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>Turret Zoom</t>
+          <t>Interaction Mode Zoom Out</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -5442,7 +5442,7 @@
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>Select Left Head</t>
+          <t>Left</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -6691,7 +6691,7 @@
       </c>
       <c r="B132" s="2" t="inlineStr">
         <is>
-          <t>Camera (3rd Person)</t>
+          <t>Enable / Disable Head Tracking for 3rd Person Camera</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
@@ -6797,7 +6797,7 @@
       </c>
       <c r="B134" s="2" t="inlineStr">
         <is>
-          <t>Head Tracking On/Off</t>
+          <t>Recenter Head Tracking Device (except TrackIR)</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
@@ -6850,7 +6850,7 @@
       </c>
       <c r="B135" s="2" t="inlineStr">
         <is>
-          <t>Select Left Head</t>
+          <t>Roll Left (while Prone)</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
@@ -6903,7 +6903,7 @@
       </c>
       <c r="B136" s="2" t="inlineStr">
         <is>
-          <t>Cycle Right Tool</t>
+          <t>Roll Right (while Prone)</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
@@ -7001,7 +7001,7 @@
       </c>
       <c r="B138" s="2" t="inlineStr">
         <is>
-          <t>Exit Seat</t>
+          <t>Emergency Exit Seat</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
@@ -7054,7 +7054,7 @@
       </c>
       <c r="B139" s="2" t="inlineStr">
         <is>
-          <t>Next Remote Turret*</t>
+          <t>Enter Remote Turret 1</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
@@ -7107,7 +7107,7 @@
       </c>
       <c r="B140" s="2" t="inlineStr">
         <is>
-          <t>Next Remote Turret*</t>
+          <t>Enter Remote Turret 2</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
@@ -7160,7 +7160,7 @@
       </c>
       <c r="B141" s="2" t="inlineStr">
         <is>
-          <t>Next Remote Turret*</t>
+          <t>Enter Remote Turret 3</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
@@ -7213,7 +7213,7 @@
       </c>
       <c r="B142" s="2" t="inlineStr">
         <is>
-          <t>Light Ampliﬁcation Toggle</t>
+          <t>Light Ampliﬁcation</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
@@ -7262,7 +7262,7 @@
       <c r="A143" t="inlineStr"/>
       <c r="B143" s="2" t="inlineStr">
         <is>
-          <t>Guns Toggle</t>
+          <t>Guns</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
@@ -7303,7 +7303,7 @@
       <c r="A144" t="inlineStr"/>
       <c r="B144" s="2" t="inlineStr">
         <is>
-          <t>Missile Cinematic Camera Toggle</t>
+          <t>Missile Mode Toggle</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
@@ -7352,7 +7352,7 @@
       <c r="A145" t="inlineStr"/>
       <c r="B145" s="2" t="inlineStr">
         <is>
-          <t>Salvage Gimbal Toggle</t>
+          <t>Salvage Mode Toggle</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
@@ -7401,7 +7401,7 @@
       </c>
       <c r="B146" s="2" t="inlineStr">
         <is>
-          <t>Look Behind</t>
+          <t>Look behind</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
@@ -7446,7 +7446,7 @@
       <c r="A147" t="inlineStr"/>
       <c r="B147" s="2" t="inlineStr">
         <is>
-          <t>Cycle MFD Page Forward</t>
+          <t>View Cycle Fwd</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
@@ -7552,7 +7552,7 @@
       </c>
       <c r="B149" s="2" t="inlineStr">
         <is>
-          <t>Shield Cap Increase</t>
+          <t>Shield raise level bottom</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
@@ -7605,7 +7605,7 @@
       </c>
       <c r="B150" s="2" t="inlineStr">
         <is>
-          <t>Shield Cap Increase</t>
+          <t>Shield raise level front</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
@@ -7658,7 +7658,7 @@
       </c>
       <c r="B151" s="2" t="inlineStr">
         <is>
-          <t>Shield Cap Increase</t>
+          <t>Shield raise level left</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
@@ -7711,7 +7711,7 @@
       </c>
       <c r="B152" s="2" t="inlineStr">
         <is>
-          <t>Shield Cap Increase</t>
+          <t>Shield raise level right</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
@@ -7764,7 +7764,7 @@
       </c>
       <c r="B153" s="2" t="inlineStr">
         <is>
-          <t>Shield Cap Increase</t>
+          <t>Shield raise level top</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
@@ -7817,7 +7817,7 @@
       </c>
       <c r="B154" s="2" t="inlineStr">
         <is>
-          <t>Shield Cap Increase</t>
+          <t>Shield reset levels</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
@@ -7976,7 +7976,7 @@
       </c>
       <c r="B157" s="2" t="inlineStr">
         <is>
-          <t>Decoy Burst Size Dec</t>
+          <t>Launch Burst , Set and Launch Burst</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
@@ -8131,7 +8131,7 @@
       </c>
       <c r="B160" s="2" t="inlineStr">
         <is>
-          <t>Invoke Docking</t>
+          <t>Invoke Docking Toggle</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
@@ -8290,7 +8290,7 @@
       </c>
       <c r="B163" s="2" t="inlineStr">
         <is>
-          <t>L-THROTTLE</t>
+          <t>Inc. Cooler Rate</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
@@ -8339,7 +8339,7 @@
       <c r="A164" t="inlineStr"/>
       <c r="B164" s="2" t="inlineStr">
         <is>
-          <t>Adv.HUD Toggle</t>
+          <t>HUD Cancel</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
@@ -8384,7 +8384,7 @@
       <c r="A165" t="inlineStr"/>
       <c r="B165" s="2" t="inlineStr">
         <is>
-          <t>Adv.HUD Toggle</t>
+          <t>HUD Confirm</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
@@ -8429,7 +8429,7 @@
       <c r="A166" t="inlineStr"/>
       <c r="B166" s="2" t="inlineStr">
         <is>
-          <t>Cycle MFD Page Backward</t>
+          <t>HUD Focused Cycle Mode Back</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
@@ -8478,7 +8478,7 @@
       <c r="A167" t="inlineStr"/>
       <c r="B167" s="2" t="inlineStr">
         <is>
-          <t>Cycle MFD Page Forward</t>
+          <t>HUD Focused Cycle Mode Fwd</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
@@ -8527,7 +8527,7 @@
       <c r="A168" t="inlineStr"/>
       <c r="B168" s="2" t="inlineStr">
         <is>
-          <t>Adv.HUD Toggle</t>
+          <t>HUD Interact Toggle</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
@@ -8572,7 +8572,7 @@
       <c r="A169" t="inlineStr"/>
       <c r="B169" s="2" t="inlineStr">
         <is>
-          <t>Adv.HUD Toggle</t>
+          <t>HUD Left Panel Down</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
@@ -8621,7 +8621,7 @@
       <c r="A170" t="inlineStr"/>
       <c r="B170" s="2" t="inlineStr">
         <is>
-          <t>Adv.HUD Toggle</t>
+          <t>HUD Left Panel Left</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
@@ -8670,7 +8670,7 @@
       <c r="A171" t="inlineStr"/>
       <c r="B171" s="2" t="inlineStr">
         <is>
-          <t>Adv.HUD Toggle</t>
+          <t>HUD Left Panel Right</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
@@ -8719,7 +8719,7 @@
       <c r="A172" t="inlineStr"/>
       <c r="B172" s="2" t="inlineStr">
         <is>
-          <t>Adv.HUD Toggle</t>
+          <t>HUD Left Panel Up</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="B173" s="2" t="inlineStr">
         <is>
-          <t>Adv.HUD Toggle</t>
+          <t>Scoreboard</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
@@ -8931,7 +8931,7 @@
       </c>
       <c r="B176" s="2" t="inlineStr">
         <is>
-          <t>Dec. Mining Laser Power (Slow)</t>
+          <t>Inc. / Dec. Mining Laser Power</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
@@ -9037,7 +9037,7 @@
       </c>
       <c r="B178" s="2" t="inlineStr">
         <is>
-          <t>Mining Module 2</t>
+          <t>Activate Mining Module (Slot 2)</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
@@ -9090,7 +9090,7 @@
       </c>
       <c r="B179" s="2" t="inlineStr">
         <is>
-          <t>Mining Module 2</t>
+          <t>Activate Mining Module (Slot 3)</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
@@ -9196,7 +9196,7 @@
       </c>
       <c r="B181" s="2" t="inlineStr">
         <is>
-          <t>Fire Mining Laser Toggle</t>
+          <t>Fire Mining Laser</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
@@ -9249,7 +9249,7 @@
       </c>
       <c r="B182" s="2" t="inlineStr">
         <is>
-          <t>Mining Laser PWR ABS Toggle</t>
+          <t>Switch Mining Laser</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
@@ -9718,7 +9718,7 @@
       </c>
       <c r="B191" s="2" t="inlineStr">
         <is>
-          <t>Weapon Set to Max</t>
+          <t>Inc. Number of Armed Missiles</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
@@ -9771,7 +9771,7 @@
       </c>
       <c r="B192" s="2" t="inlineStr">
         <is>
-          <t>Missile Cinematic Camera</t>
+          <t>Launch Missiles</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
@@ -9820,7 +9820,7 @@
       <c r="A193" t="inlineStr"/>
       <c r="B193" s="2" t="inlineStr">
         <is>
-          <t>Missile Cinematic Camera</t>
+          <t>Weapon Launch Missile Cinematic</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
@@ -9873,7 +9873,7 @@
       </c>
       <c r="B194" s="2" t="inlineStr">
         <is>
-          <t>Weapon Set to Max</t>
+          <t>Reset Number of Armed Missiles</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
@@ -10032,7 +10032,7 @@
       </c>
       <c r="B197" s="2" t="inlineStr">
         <is>
-          <t>Dec. Bomb Range</t>
+          <t>Acceleration Limiter - Dec.</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
@@ -10085,7 +10085,7 @@
       </c>
       <c r="B198" s="2" t="inlineStr">
         <is>
-          <t>Inc. Bomb Range</t>
+          <t>Acceleration Limiter - Inc.</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
@@ -10326,7 +10326,7 @@
       </c>
       <c r="B203" s="2" t="inlineStr">
         <is>
-          <t>Request Landing</t>
+          <t>Landing System (Deploy)</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
@@ -10379,7 +10379,7 @@
       </c>
       <c r="B204" s="2" t="inlineStr">
         <is>
-          <t>Adv.HUD Toggle</t>
+          <t>Advanced HUD - Toggle</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
@@ -10432,7 +10432,7 @@
       </c>
       <c r="B205" s="2" t="inlineStr">
         <is>
-          <t>Speed Limiter Inc. Step</t>
+          <t>Speed Limiter ABS.</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
@@ -10485,7 +10485,7 @@
       </c>
       <c r="B206" s="2" t="inlineStr">
         <is>
-          <t>Speed Limiter Inc. Step</t>
+          <t>Speed Limiter - Step Down</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
@@ -10538,7 +10538,7 @@
       </c>
       <c r="B207" s="2" t="inlineStr">
         <is>
-          <t>Speed Limiter Inc. Step</t>
+          <t>Speed Limiter - Dec.</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
@@ -10591,7 +10591,7 @@
       </c>
       <c r="B208" s="2" t="inlineStr">
         <is>
-          <t>Speed Limiter Inc. Step</t>
+          <t>Speed Limiter - Step Up</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
@@ -10644,7 +10644,7 @@
       </c>
       <c r="B209" s="2" t="inlineStr">
         <is>
-          <t>Speed Limiter Inc. Step Toggle</t>
+          <t>Speed Limiter - Enable / Disable</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
@@ -10697,7 +10697,7 @@
       </c>
       <c r="B210" s="2" t="inlineStr">
         <is>
-          <t>Speed Limiter Inc. Step</t>
+          <t>Speed Limiter - Inc.</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
@@ -10803,7 +10803,7 @@
       </c>
       <c r="B212" s="2" t="inlineStr">
         <is>
-          <t>Cruise Control Toggle</t>
+          <t>Cruise Mode - Toggle</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
@@ -10909,7 +10909,7 @@
       </c>
       <c r="B214" s="2" t="inlineStr">
         <is>
-          <t>Power On/Off Toggle</t>
+          <t>G-Force Safety On/Off</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
@@ -11256,7 +11256,7 @@
       </c>
       <c r="B221" s="2" t="inlineStr">
         <is>
-          <t>Select Left Head</t>
+          <t>Roll left</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
@@ -11309,7 +11309,7 @@
       </c>
       <c r="B222" s="2" t="inlineStr">
         <is>
-          <t>Cycle Right Tool</t>
+          <t>Roll right</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
@@ -11411,7 +11411,7 @@
       </c>
       <c r="B224" s="2" t="inlineStr">
         <is>
-          <t>Mining Laser PWR ABS</t>
+          <t>Strafe down (abs.)</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
@@ -11464,7 +11464,7 @@
       </c>
       <c r="B225" s="2" t="inlineStr">
         <is>
-          <t>Mining Laser PWR ABS</t>
+          <t>Strafe left / right (abs.)</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
@@ -11517,7 +11517,7 @@
       </c>
       <c r="B226" s="2" t="inlineStr">
         <is>
-          <t>Mining Laser PWR ABS</t>
+          <t>Strafe left (abs.)</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
@@ -11570,7 +11570,7 @@
       </c>
       <c r="B227" s="2" t="inlineStr">
         <is>
-          <t>L-THROTTLE</t>
+          <t>Forward / Back</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
@@ -11623,7 +11623,7 @@
       </c>
       <c r="B228" s="2" t="inlineStr">
         <is>
-          <t>L-THROTTLE</t>
+          <t>Forward / Back Invert</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
@@ -11676,7 +11676,7 @@
       </c>
       <c r="B229" s="2" t="inlineStr">
         <is>
-          <t>Mining Laser PWR ABS</t>
+          <t>Strafe right (abs.)</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
@@ -11888,7 +11888,7 @@
       </c>
       <c r="B233" s="2" t="inlineStr">
         <is>
-          <t>L-THROTTLE</t>
+          <t>Trim - Set To 50%</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
@@ -11941,7 +11941,7 @@
       </c>
       <c r="B234" s="2" t="inlineStr">
         <is>
-          <t>L-THROTTLE</t>
+          <t>Trim - Set To 50%</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
@@ -11994,7 +11994,7 @@
       </c>
       <c r="B235" s="2" t="inlineStr">
         <is>
-          <t>L-THROTTLE</t>
+          <t>Trim - Set</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
@@ -12047,7 +12047,7 @@
       </c>
       <c r="B236" s="2" t="inlineStr">
         <is>
-          <t>Mining Laser PWR ABS</t>
+          <t>Strafe up (abs.)</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
@@ -12100,7 +12100,7 @@
       </c>
       <c r="B237" s="2" t="inlineStr">
         <is>
-          <t>Mining Laser PWR ABS</t>
+          <t>Strafe up / down (abs.)</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
@@ -12153,7 +12153,7 @@
       </c>
       <c r="B238" s="2" t="inlineStr">
         <is>
-          <t>Request Landing Toggle</t>
+          <t>Jump Drive - Request Jump</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
@@ -12206,7 +12206,7 @@
       </c>
       <c r="B239" s="2" t="inlineStr">
         <is>
-          <t>Swap Yaw / Roll Toggle</t>
+          <t>Swap Yaw / Roll</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
@@ -12329,7 +12329,7 @@
       </c>
       <c r="B242" s="2" t="inlineStr">
         <is>
-          <t>Retract Conﬁg</t>
+          <t>Retract Configuration</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
@@ -12366,7 +12366,7 @@
       <c r="A243" t="inlineStr"/>
       <c r="B243" s="2" t="inlineStr">
         <is>
-          <t>VTOL Toggle</t>
+          <t>VTOL Off</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
@@ -12415,7 +12415,7 @@
       <c r="A244" t="inlineStr"/>
       <c r="B244" s="2" t="inlineStr">
         <is>
-          <t>VTOL Toggle</t>
+          <t>VTOL On</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
@@ -12640,7 +12640,7 @@
       <c r="A249" t="inlineStr"/>
       <c r="B249" s="2" t="inlineStr">
         <is>
-          <t>Capacitor Reset</t>
+          <t>Engineering Assignment Engine Min</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
@@ -12787,7 +12787,7 @@
       </c>
       <c r="B252" s="2" t="inlineStr">
         <is>
-          <t>Shields Power Toggle</t>
+          <t>Shields Inc.</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
@@ -12938,7 +12938,7 @@
       </c>
       <c r="B255" s="2" t="inlineStr">
         <is>
-          <t>Dec.</t>
+          <t>Weapons Dec.</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
@@ -12979,7 +12979,7 @@
       </c>
       <c r="B256" s="2" t="inlineStr">
         <is>
-          <t>Inc.</t>
+          <t>Weapons Inc.</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
@@ -13016,7 +13016,7 @@
       <c r="A257" t="inlineStr"/>
       <c r="B257" s="2" t="inlineStr">
         <is>
-          <t>Weapon Set to Max</t>
+          <t>Engineering Assignment Weapons Max</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
@@ -13118,7 +13118,7 @@
       </c>
       <c r="B259" s="2" t="inlineStr">
         <is>
-          <t>Inc. Mining Laser Power (Slow)</t>
+          <t>Inc. Throttle to Max</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
@@ -13171,7 +13171,7 @@
       </c>
       <c r="B260" s="2" t="inlineStr">
         <is>
-          <t>Dec. Mining Laser Power (Slow)</t>
+          <t>Dec. Throttle to Min</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
@@ -13224,7 +13224,7 @@
       </c>
       <c r="B261" s="2" t="inlineStr">
         <is>
-          <t>Weapon Power Toggle</t>
+          <t>Power - All Toggle</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
@@ -13277,7 +13277,7 @@
       </c>
       <c r="B262" s="2" t="inlineStr">
         <is>
-          <t>Shields Power Toggle</t>
+          <t>Power - Shields Toggle</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
@@ -13330,7 +13330,7 @@
       </c>
       <c r="B263" s="2" t="inlineStr">
         <is>
-          <t>Weapon Power Toggle</t>
+          <t>Power - Thrusters Toggle</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
@@ -13383,7 +13383,7 @@
       </c>
       <c r="B264" s="2" t="inlineStr">
         <is>
-          <t>Weapon Power Toggle</t>
+          <t>Power - Weapons Toggle</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
@@ -13436,7 +13436,7 @@
       </c>
       <c r="B265" s="2" t="inlineStr">
         <is>
-          <t>Engage Quantum Toggle</t>
+          <t>Engage Quantum</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
@@ -13538,7 +13538,7 @@
       <c r="A267" t="inlineStr"/>
       <c r="B267" s="2" t="inlineStr">
         <is>
-          <t>Dec. Tractor Distance</t>
+          <t>Tractor Beam Vehicle Dec. Distance</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
@@ -13587,7 +13587,7 @@
       <c r="A268" t="inlineStr"/>
       <c r="B268" s="2" t="inlineStr">
         <is>
-          <t>Tractor Distance Inc.</t>
+          <t>Tractor Beam Vehicle Inc. Distance</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
@@ -13746,7 +13746,7 @@
       </c>
       <c r="B271" s="2" t="inlineStr">
         <is>
-          <t>Cycle Right Tool</t>
+          <t>Cycle Right Salvage Modifiers</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
@@ -13893,7 +13893,7 @@
       <c r="A274" t="inlineStr"/>
       <c r="B274" s="2" t="inlineStr">
         <is>
-          <t>Focus All Salvage Heads</t>
+          <t>Salvage Focus Disintegrate</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
@@ -13991,7 +13991,7 @@
       <c r="A276" t="inlineStr"/>
       <c r="B276" s="2" t="inlineStr">
         <is>
-          <t>Focus Left Tool</t>
+          <t>Salvage Focus Left</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
@@ -14040,7 +14040,7 @@
       <c r="A277" t="inlineStr"/>
       <c r="B277" s="2" t="inlineStr">
         <is>
-          <t>Focus Right Tool</t>
+          <t>Salvage Focus Right</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
@@ -14146,7 +14146,7 @@
       </c>
       <c r="B279" s="2" t="inlineStr">
         <is>
-          <t>Salvage Beam Spacing Toggle</t>
+          <t>Salvage Beam Axis</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
@@ -14195,7 +14195,7 @@
       <c r="A280" t="inlineStr"/>
       <c r="B280" s="2" t="inlineStr">
         <is>
-          <t>Fire Fracture Toggle</t>
+          <t>Fire Fracture</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
@@ -14244,7 +14244,7 @@
       <c r="A281" t="inlineStr"/>
       <c r="B281" s="2" t="inlineStr">
         <is>
-          <t>Fire Left Tool Toggle</t>
+          <t>Fire Left Tool</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
@@ -14293,7 +14293,7 @@
       <c r="A282" t="inlineStr"/>
       <c r="B282" s="2" t="inlineStr">
         <is>
-          <t>Fire Right Tool Toggle</t>
+          <t>Salvage Fire Right Toggle</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
@@ -14505,7 +14505,7 @@
       </c>
       <c r="B286" s="2" t="inlineStr">
         <is>
-          <t>Scan Ping</t>
+          <t>Activate Scanning</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
@@ -14607,7 +14607,7 @@
       </c>
       <c r="B288" s="2" t="inlineStr">
         <is>
-          <t>Power On/Off Toggle</t>
+          <t>Auto Targeting - On/Off Toggle</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
@@ -14660,7 +14660,7 @@
       </c>
       <c r="B289" s="2" t="inlineStr">
         <is>
-          <t>Look Behind</t>
+          <t>Enable / Disable Look Ahead</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
@@ -14709,7 +14709,7 @@
       </c>
       <c r="B290" s="2" t="inlineStr">
         <is>
-          <t>Look Behind</t>
+          <t>Enable / Disable Target Padlock (Toggle, Hold)</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
@@ -14868,7 +14868,7 @@
       </c>
       <c r="B293" s="2" t="inlineStr">
         <is>
-          <t>Unlock Current Target Toggle</t>
+          <t>Unlock Current Target</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
@@ -14921,7 +14921,7 @@
       </c>
       <c r="B294" s="2" t="inlineStr">
         <is>
-          <t>Unlock Current Target Toggle</t>
+          <t>Pin Index 2 - Lock / Unlock Pinned Target</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
@@ -14974,7 +14974,7 @@
       </c>
       <c r="B295" s="2" t="inlineStr">
         <is>
-          <t>Unlock Current Target Toggle</t>
+          <t>Pin Index 3 - Lock / Unlock Pinned Target</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
@@ -15027,7 +15027,7 @@
       </c>
       <c r="B296" s="2" t="inlineStr">
         <is>
-          <t>Pin/Unpin 2 Toggle</t>
+          <t>Pin/Unpin 2</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
@@ -15080,7 +15080,7 @@
       </c>
       <c r="B297" s="2" t="inlineStr">
         <is>
-          <t>Pin/Unpin 2 Toggle</t>
+          <t>Pin Index 1 - Pin / Unpin Selected Target</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
@@ -15133,7 +15133,7 @@
       </c>
       <c r="B298" s="2" t="inlineStr">
         <is>
-          <t>Pin/Unpin 2 Toggle</t>
+          <t>Pin Index 2 - Pin / Unpin Selected Target</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
@@ -15186,7 +15186,7 @@
       </c>
       <c r="B299" s="2" t="inlineStr">
         <is>
-          <t>Pin/Unpin 2 Toggle</t>
+          <t>Pin Index 2 - Pin / Unpin Selected Target</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
@@ -15239,7 +15239,7 @@
       </c>
       <c r="B300" s="2" t="inlineStr">
         <is>
-          <t>Pin/Unpin 2 Toggle</t>
+          <t>Pin Index 3 - Pin / Unpin Selected Target</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
@@ -15292,7 +15292,7 @@
       </c>
       <c r="B301" s="2" t="inlineStr">
         <is>
-          <t>Pin/Unpin 2 Toggle</t>
+          <t>Pin Index 3 - Pin / Unpin Selected Target</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
@@ -15875,7 +15875,7 @@
       </c>
       <c r="B312" s="2" t="inlineStr">
         <is>
-          <t>Target Under Reticle</t>
+          <t>Lock Target Under Reticle</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
@@ -15924,7 +15924,7 @@
       <c r="A313" t="inlineStr"/>
       <c r="B313" s="2" t="inlineStr">
         <is>
-          <t>ADS Zoom Toggle</t>
+          <t>ADS</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
@@ -15965,7 +15965,7 @@
       <c r="A314" t="inlineStr"/>
       <c r="B314" s="2" t="inlineStr">
         <is>
-          <t>ADS Zoom Toggle</t>
+          <t>ADS Stable Max Zoom</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -16014,7 +16014,7 @@
       <c r="A315" t="inlineStr"/>
       <c r="B315" s="2" t="inlineStr">
         <is>
-          <t>Cycle MFD Page Forward</t>
+          <t>View Cycle Internal Fwd</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
@@ -16067,7 +16067,7 @@
       </c>
       <c r="B316" s="2" t="inlineStr">
         <is>
-          <t>Missile Cinematic Camera</t>
+          <t>Cycle camera orbit mode</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
@@ -16120,7 +16120,7 @@
       </c>
       <c r="B317" s="2" t="inlineStr">
         <is>
-          <t>Look Behind</t>
+          <t>Look down</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
@@ -16173,7 +16173,7 @@
       </c>
       <c r="B318" s="2" t="inlineStr">
         <is>
-          <t>Look Behind</t>
+          <t>Look up</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
@@ -16226,7 +16226,7 @@
       </c>
       <c r="B319" s="2" t="inlineStr">
         <is>
-          <t>Look Behind</t>
+          <t>Look left</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
@@ -16279,7 +16279,7 @@
       </c>
       <c r="B320" s="2" t="inlineStr">
         <is>
-          <t>Look Behind</t>
+          <t>Look right</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
@@ -16332,7 +16332,7 @@
       </c>
       <c r="B321" s="2" t="inlineStr">
         <is>
-          <t>Missile Type Previous</t>
+          <t>AIM Mode - Cycle</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
@@ -16385,7 +16385,7 @@
       </c>
       <c r="B322" s="2" t="inlineStr">
         <is>
-          <t>Missile Type Previous</t>
+          <t>AIM Mode - Set to Painting</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
@@ -16491,7 +16491,7 @@
       </c>
       <c r="B324" s="2" t="inlineStr">
         <is>
-          <t>Salvage Gimbal Toggle</t>
+          <t>Gimbal State - Locked / Unlocked Toggle</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
@@ -16597,7 +16597,7 @@
       </c>
       <c r="B326" s="2" t="inlineStr">
         <is>
-          <t>Prev. Weapon Preset</t>
+          <t>Weapon Preset - Fire</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
@@ -16756,7 +16756,7 @@
       </c>
       <c r="B329" s="2" t="inlineStr">
         <is>
-          <t>Fire Selected Weapon Group</t>
+          <t>Weapon Presets - Fire Guns Group 2</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
@@ -16809,7 +16809,7 @@
       </c>
       <c r="B330" s="2" t="inlineStr">
         <is>
-          <t>Fire Selected Weapon Group</t>
+          <t>Weapon Presets - Fire Guns Group 3</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
@@ -16862,7 +16862,7 @@
       </c>
       <c r="B331" s="2" t="inlineStr">
         <is>
-          <t>Fire Selected Weapon Group</t>
+          <t>Weapon Presets - Fire Guns Group 4</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
@@ -16915,7 +16915,7 @@
       </c>
       <c r="B332" s="2" t="inlineStr">
         <is>
-          <t>Fire Selected Weapon Group</t>
+          <t>Weapon Presets - Set Guns Group 1</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
@@ -16968,7 +16968,7 @@
       </c>
       <c r="B333" s="2" t="inlineStr">
         <is>
-          <t>Fire Selected Weapon Group</t>
+          <t>Weapon Presets - Set Guns Group 2</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
@@ -17021,7 +17021,7 @@
       </c>
       <c r="B334" s="2" t="inlineStr">
         <is>
-          <t>Prev. Weapon Preset</t>
+          <t>Weapon Presets - Prev.</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
@@ -17074,7 +17074,7 @@
       </c>
       <c r="B335" s="2" t="inlineStr">
         <is>
-          <t>Prev. Weapon Preset</t>
+          <t>Prev. Weapon Preset (Overflow)</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
@@ -17127,7 +17127,7 @@
       </c>
       <c r="B336" s="2" t="inlineStr">
         <is>
-          <t>EMP/QID Preset</t>
+          <t>Weapon Presets - Set QIDs</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
@@ -17180,7 +17180,7 @@
       </c>
       <c r="B337" s="2" t="inlineStr">
         <is>
-          <t>EMP/QID Preset</t>
+          <t>Weapon Presets - Set Quantum Jammers (short range)</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
@@ -17233,7 +17233,7 @@
       </c>
       <c r="B338" s="2" t="inlineStr">
         <is>
-          <t>EMP/QID Preset</t>
+          <t>Weapon Presets - Set Quantum Snares / Pulse (long range)</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
@@ -17286,7 +17286,7 @@
       </c>
       <c r="B339" s="2" t="inlineStr">
         <is>
-          <t>Power On/Off Toggle</t>
+          <t>Staggered Fire - On / Off Toggle</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
@@ -17335,7 +17335,7 @@
       <c r="A340" t="inlineStr"/>
       <c r="B340" s="2" t="inlineStr">
         <is>
-          <t>Look Behind</t>
+          <t>Spectate Free Look</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
@@ -17384,7 +17384,7 @@
       </c>
       <c r="B341" s="2" t="inlineStr">
         <is>
-          <t>Next Remote Turret*</t>
+          <t>Spectator Camera Target (Next)</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
@@ -17437,7 +17437,7 @@
       </c>
       <c r="B342" s="2" t="inlineStr">
         <is>
-          <t>Previous Remote Turret*</t>
+          <t>Spectator Camera Target (Prev.)</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
@@ -17490,7 +17490,7 @@
       </c>
       <c r="B343" s="2" t="inlineStr">
         <is>
-          <t>Missile Cinematic Camera</t>
+          <t>Spectator Camera Rotate Pitch</t>
         </is>
       </c>
       <c r="C343" t="inlineStr">
@@ -17596,7 +17596,7 @@
       </c>
       <c r="B345" s="2" t="inlineStr">
         <is>
-          <t>Missile Cinematic Camera</t>
+          <t>Spectator Camera Rotate Yaw</t>
         </is>
       </c>
       <c r="C345" t="inlineStr">
@@ -17649,7 +17649,7 @@
       </c>
       <c r="B346" s="2" t="inlineStr">
         <is>
-          <t>Turret Mouse Mode*</t>
+          <t>Spectator Camera Rotate Yaw</t>
         </is>
       </c>
       <c r="C346" t="inlineStr">
@@ -17698,7 +17698,7 @@
       <c r="A347" t="inlineStr"/>
       <c r="B347" s="2" t="inlineStr">
         <is>
-          <t>Speed Limiter Inc. Step</t>
+          <t>Spectate Speed Decrement</t>
         </is>
       </c>
       <c r="C347" t="inlineStr">
@@ -17739,7 +17739,7 @@
       <c r="A348" t="inlineStr"/>
       <c r="B348" s="2" t="inlineStr">
         <is>
-          <t>Speed Limiter Inc. Step</t>
+          <t>Spectate Speed Increment</t>
         </is>
       </c>
       <c r="C348" t="inlineStr">
@@ -17784,7 +17784,7 @@
       </c>
       <c r="B349" s="2" t="inlineStr">
         <is>
-          <t>Missile Cinematic Camera</t>
+          <t>Spectator Camera Zoom</t>
         </is>
       </c>
       <c r="C349" t="inlineStr">
@@ -17837,7 +17837,7 @@
       </c>
       <c r="B350" s="2" t="inlineStr">
         <is>
-          <t>Missile Cinematic Camera</t>
+          <t>Spectator Camera Zoom In</t>
         </is>
       </c>
       <c r="C350" t="inlineStr">
@@ -17890,7 +17890,7 @@
       </c>
       <c r="B351" s="2" t="inlineStr">
         <is>
-          <t>Missile Cinematic Camera</t>
+          <t>Spectator Camera Zoom Out</t>
         </is>
       </c>
       <c r="C351" t="inlineStr">
@@ -17984,7 +17984,7 @@
       </c>
       <c r="B353" s="2" t="inlineStr">
         <is>
-          <t>Start/Pause Stop Watch</t>
+          <t>Start / Pause</t>
         </is>
       </c>
       <c r="C353" t="inlineStr">
@@ -18192,7 +18192,7 @@
       </c>
       <c r="B357" s="2" t="inlineStr">
         <is>
-          <t>Power On/Off Toggle</t>
+          <t>Turret E.S.P. On / Off Toggle</t>
         </is>
       </c>
       <c r="C357" t="inlineStr">
@@ -18245,7 +18245,7 @@
       </c>
       <c r="B358" s="2" t="inlineStr">
         <is>
-          <t>Speed Limiter Inc. Step</t>
+          <t>Turret - Speed Limiter ABS.</t>
         </is>
       </c>
       <c r="C358" t="inlineStr">
@@ -18298,7 +18298,7 @@
       </c>
       <c r="B359" s="2" t="inlineStr">
         <is>
-          <t>Speed Limiter Inc. Step</t>
+          <t>Turret - Speed Limiter REL.</t>
         </is>
       </c>
       <c r="C359" t="inlineStr">
@@ -18351,7 +18351,7 @@
       </c>
       <c r="B360" s="2" t="inlineStr">
         <is>
-          <t>Speed Limiter Inc. Step</t>
+          <t>Turret - Speed Limiter - Dec. REL.</t>
         </is>
       </c>
       <c r="C360" t="inlineStr">
@@ -18404,7 +18404,7 @@
       </c>
       <c r="B361" s="2" t="inlineStr">
         <is>
-          <t>Speed Limiter Inc. Step</t>
+          <t>Turret - Speed Limiter - Inc. REL.</t>
         </is>
       </c>
       <c r="C361" t="inlineStr">
@@ -18457,7 +18457,7 @@
       </c>
       <c r="B362" s="2" t="inlineStr">
         <is>
-          <t>Speed Limiter Inc. Step Toggle</t>
+          <t>Turret - Speed Limiter - On/Off (Hold/Toggle)</t>
         </is>
       </c>
       <c r="C362" t="inlineStr">
@@ -18649,7 +18649,7 @@
       </c>
       <c r="B366" s="2" t="inlineStr">
         <is>
-          <t>Turret VJOY* Toggle</t>
+          <t>Turret VJOY*</t>
         </is>
       </c>
       <c r="C366" t="inlineStr">
@@ -18743,7 +18743,7 @@
       </c>
       <c r="B368" s="2" t="inlineStr">
         <is>
-          <t>Space Brake</t>
+          <t>Brake</t>
         </is>
       </c>
       <c r="C368" t="inlineStr">
@@ -18784,7 +18784,7 @@
       </c>
       <c r="B369" s="2" t="inlineStr">
         <is>
-          <t>Cycle MFD Page Backward</t>
+          <t>Drive Forward / Backward</t>
         </is>
       </c>
       <c r="C369" t="inlineStr">
@@ -18837,7 +18837,7 @@
       </c>
       <c r="B370" s="2" t="inlineStr">
         <is>
-          <t>Cycle MFD Page Backward</t>
+          <t>Drive Backward</t>
         </is>
       </c>
       <c r="C370" t="inlineStr">
@@ -18890,7 +18890,7 @@
       </c>
       <c r="B371" s="2" t="inlineStr">
         <is>
-          <t>Cycle MFD Page Forward</t>
+          <t>Drive Forward</t>
         </is>
       </c>
       <c r="C371" t="inlineStr">
@@ -19049,7 +19049,7 @@
       </c>
       <c r="B374" s="2" t="inlineStr">
         <is>
-          <t>Turret Mouse Mode*</t>
+          <t>Pitch Up / Down (Mouse)</t>
         </is>
       </c>
       <c r="C374" t="inlineStr">
@@ -19208,7 +19208,7 @@
       </c>
       <c r="B377" s="2" t="inlineStr">
         <is>
-          <t>Dynamic Zoom Toggle</t>
+          <t>Dynamic Zoom (abs.) Toggle</t>
         </is>
       </c>
       <c r="C377" t="inlineStr">
@@ -19261,7 +19261,7 @@
       </c>
       <c r="B378" s="2" t="inlineStr">
         <is>
-          <t>Dynamic Zoom</t>
+          <t>Dynamic Zoom In and Out (rel.)</t>
         </is>
       </c>
       <c r="C378" t="inlineStr">
@@ -19314,7 +19314,7 @@
       </c>
       <c r="B379" s="2" t="inlineStr">
         <is>
-          <t>Dynamic Zoom</t>
+          <t>Dynamic Zoom In (rel.)</t>
         </is>
       </c>
       <c r="C379" t="inlineStr">
@@ -19367,7 +19367,7 @@
       </c>
       <c r="B380" s="2" t="inlineStr">
         <is>
-          <t>Dynamic Zoom</t>
+          <t>Dynamic Zoom Out (rel.)</t>
         </is>
       </c>
       <c r="C380" t="inlineStr">
@@ -19420,7 +19420,7 @@
       </c>
       <c r="B381" s="2" t="inlineStr">
         <is>
-          <t>Beam Axis Toggle</t>
+          <t>Yaw Left / Right (Axis / HOTAS)</t>
         </is>
       </c>
       <c r="C381" t="inlineStr">
@@ -19473,7 +19473,7 @@
       </c>
       <c r="B382" s="2" t="inlineStr">
         <is>
-          <t>Select Left Head</t>
+          <t>Turn Left</t>
         </is>
       </c>
       <c r="C382" t="inlineStr">
@@ -19526,7 +19526,7 @@
       </c>
       <c r="B383" s="2" t="inlineStr">
         <is>
-          <t>Turret Mouse Mode*</t>
+          <t>Yaw Left / Right (Mouse)</t>
         </is>
       </c>
       <c r="C383" t="inlineStr">
@@ -19579,7 +19579,7 @@
       </c>
       <c r="B384" s="2" t="inlineStr">
         <is>
-          <t>Cycle Right Tool</t>
+          <t>Turn Right</t>
         </is>
       </c>
       <c r="C384" t="inlineStr">
@@ -19779,7 +19779,7 @@
       </c>
       <c r="B388" s="2" t="inlineStr">
         <is>
-          <t>Lock Doors</t>
+          <t>Lock All Doors</t>
         </is>
       </c>
       <c r="C388" t="inlineStr">
@@ -20085,7 +20085,7 @@
       </c>
       <c r="B394" s="2" t="inlineStr">
         <is>
-          <t>Unlock Doors</t>
+          <t>Port Unlock All</t>
         </is>
       </c>
       <c r="C394" t="inlineStr">
@@ -20191,7 +20191,7 @@
       </c>
       <c r="B396" s="2" t="inlineStr">
         <is>
-          <t>Look Behind</t>
+          <t>Look up / down</t>
         </is>
       </c>
       <c r="C396" t="inlineStr">
@@ -20244,7 +20244,7 @@
       </c>
       <c r="B397" s="2" t="inlineStr">
         <is>
-          <t>Look Behind</t>
+          <t>Look up / down</t>
         </is>
       </c>
       <c r="C397" t="inlineStr">
@@ -20297,7 +20297,7 @@
       </c>
       <c r="B398" s="2" t="inlineStr">
         <is>
-          <t>Look Behind</t>
+          <t>Look left / right</t>
         </is>
       </c>
       <c r="C398" t="inlineStr">
@@ -20350,7 +20350,7 @@
       </c>
       <c r="B399" s="2" t="inlineStr">
         <is>
-          <t>Look Behind</t>
+          <t>Look left / right</t>
         </is>
       </c>
       <c r="C399" t="inlineStr">
@@ -20403,7 +20403,7 @@
       </c>
       <c r="B400" s="2" t="inlineStr">
         <is>
-          <t>Camera (3rd Person)</t>
+          <t>Zoom in (3rd person view)</t>
         </is>
       </c>
       <c r="C400" t="inlineStr">
@@ -20456,7 +20456,7 @@
       </c>
       <c r="B401" s="2" t="inlineStr">
         <is>
-          <t>Camera (3rd Person)</t>
+          <t>Zoom out (3rd person view)</t>
         </is>
       </c>
       <c r="C401" t="inlineStr">
@@ -20509,7 +20509,7 @@
       </c>
       <c r="B402" s="2" t="inlineStr">
         <is>
-          <t>Cycle MFD Page Backward</t>
+          <t>Cycle Page - Backwards</t>
         </is>
       </c>
       <c r="C402" t="inlineStr">
@@ -20562,7 +20562,7 @@
       </c>
       <c r="B403" s="2" t="inlineStr">
         <is>
-          <t>Cycle MFD Page Backward</t>
+          <t>Cycle Page - Backwards</t>
         </is>
       </c>
       <c r="C403" t="inlineStr">
@@ -20615,7 +20615,7 @@
       </c>
       <c r="B404" s="2" t="inlineStr">
         <is>
-          <t>Cycle MFD Page Forward</t>
+          <t>Cycle Page - Forwards</t>
         </is>
       </c>
       <c r="C404" t="inlineStr">
@@ -20668,7 +20668,7 @@
       </c>
       <c r="B405" s="2" t="inlineStr">
         <is>
-          <t>Cycle MFD Page Forward</t>
+          <t>Cycle Page - Forwards</t>
         </is>
       </c>
       <c r="C405" t="inlineStr">
@@ -20721,7 +20721,7 @@
       </c>
       <c r="B406" s="2" t="inlineStr">
         <is>
-          <t>Select MFD Down</t>
+          <t>Movement - Down</t>
         </is>
       </c>
       <c r="C406" t="inlineStr">
@@ -20880,7 +20880,7 @@
       </c>
       <c r="B409" s="2" t="inlineStr">
         <is>
-          <t>Select MFD Up</t>
+          <t>Movement - Up</t>
         </is>
       </c>
       <c r="C409" t="inlineStr">
@@ -20933,7 +20933,7 @@
       </c>
       <c r="B410" s="2" t="inlineStr">
         <is>
-          <t>Cycle MFD Page Backward</t>
+          <t>Set Page - Communications</t>
         </is>
       </c>
       <c r="C410" t="inlineStr">
@@ -20986,7 +20986,7 @@
       </c>
       <c r="B411" s="2" t="inlineStr">
         <is>
-          <t>Cycle MFD Page Backward</t>
+          <t>Set Page - Vehicle Configuration</t>
         </is>
       </c>
       <c r="C411" t="inlineStr">
@@ -21039,7 +21039,7 @@
       </c>
       <c r="B412" s="2" t="inlineStr">
         <is>
-          <t>Cycle MFD Page Backward</t>
+          <t>Set Page - Diagnostics</t>
         </is>
       </c>
       <c r="C412" t="inlineStr">
@@ -21092,7 +21092,7 @@
       </c>
       <c r="B413" s="2" t="inlineStr">
         <is>
-          <t>Cycle MFD Page Backward</t>
+          <t>Set Page - IFCS</t>
         </is>
       </c>
       <c r="C413" t="inlineStr">
@@ -21145,7 +21145,7 @@
       </c>
       <c r="B414" s="2" t="inlineStr">
         <is>
-          <t>Cycle MFD Page Backward</t>
+          <t>Set Page - Resource Network</t>
         </is>
       </c>
       <c r="C414" t="inlineStr">
@@ -21198,7 +21198,7 @@
       </c>
       <c r="B415" s="2" t="inlineStr">
         <is>
-          <t>Cycle MFD Page Backward</t>
+          <t>Set Page - Scanning</t>
         </is>
       </c>
       <c r="C415" t="inlineStr">
@@ -21251,7 +21251,7 @@
       </c>
       <c r="B416" s="2" t="inlineStr">
         <is>
-          <t>Cycle MFD Page Backward</t>
+          <t>Set Page - Self Status</t>
         </is>
       </c>
       <c r="C416" t="inlineStr">
@@ -21304,7 +21304,7 @@
       </c>
       <c r="B417" s="2" t="inlineStr">
         <is>
-          <t>Cycle MFD Page Backward</t>
+          <t>Set Page - Target Status</t>
         </is>
       </c>
       <c r="C417" t="inlineStr">
@@ -21357,7 +21357,7 @@
       </c>
       <c r="B418" s="2" t="inlineStr">
         <is>
-          <t>Select MFD Left</t>
+          <t>Select - MFD 1</t>
         </is>
       </c>
       <c r="C418" t="inlineStr">
@@ -21410,7 +21410,7 @@
       </c>
       <c r="B419" s="2" t="inlineStr">
         <is>
-          <t>Select MFD Left</t>
+          <t>Select - MFD 2</t>
         </is>
       </c>
       <c r="C419" t="inlineStr">
@@ -21463,7 +21463,7 @@
       </c>
       <c r="B420" s="2" t="inlineStr">
         <is>
-          <t>Select MFD Left</t>
+          <t>Select - MFD 3</t>
         </is>
       </c>
       <c r="C420" t="inlineStr">
@@ -21516,7 +21516,7 @@
       </c>
       <c r="B421" s="2" t="inlineStr">
         <is>
-          <t>Select MFD Left</t>
+          <t>Select - MFD 4</t>
         </is>
       </c>
       <c r="C421" t="inlineStr">
@@ -21569,7 +21569,7 @@
       </c>
       <c r="B422" s="2" t="inlineStr">
         <is>
-          <t>Select MFD Left</t>
+          <t>Select - MFD 5</t>
         </is>
       </c>
       <c r="C422" t="inlineStr">
@@ -21622,7 +21622,7 @@
       </c>
       <c r="B423" s="2" t="inlineStr">
         <is>
-          <t>Select MFD Left</t>
+          <t>Select - MFD 6</t>
         </is>
       </c>
       <c r="C423" t="inlineStr">
@@ -21675,7 +21675,7 @@
       </c>
       <c r="B424" s="2" t="inlineStr">
         <is>
-          <t>Select MFD Left</t>
+          <t>Select - MFD 7</t>
         </is>
       </c>
       <c r="C424" t="inlineStr">
@@ -21728,7 +21728,7 @@
       </c>
       <c r="B425" s="2" t="inlineStr">
         <is>
-          <t>Select MFD Left</t>
+          <t>Select - MFD 8</t>
         </is>
       </c>
       <c r="C425" t="inlineStr">
@@ -21904,7 +21904,7 @@
       </c>
       <c r="B429" s="2" t="inlineStr">
         <is>
-          <t>Unlock Current Target</t>
+          <t>Reset Current View</t>
         </is>
       </c>
       <c r="C429" t="inlineStr">
@@ -21990,7 +21990,7 @@
       </c>
       <c r="B431" s="2" t="inlineStr">
         <is>
-          <t>Space Brake</t>
+          <t>Brake</t>
         </is>
       </c>
       <c r="C431" t="inlineStr">
@@ -22031,7 +22031,7 @@
       </c>
       <c r="B432" s="2" t="inlineStr">
         <is>
-          <t>Select Left Head</t>
+          <t>Roll Left/Right</t>
         </is>
       </c>
       <c r="C432" t="inlineStr">
@@ -22084,7 +22084,7 @@
       </c>
       <c r="B433" s="2" t="inlineStr">
         <is>
-          <t>Select Left Head</t>
+          <t>Roll Left</t>
         </is>
       </c>
       <c r="C433" t="inlineStr">
@@ -22137,7 +22137,7 @@
       </c>
       <c r="B434" s="2" t="inlineStr">
         <is>
-          <t>Cycle Right Tool</t>
+          <t>Roll Right</t>
         </is>
       </c>
       <c r="C434" t="inlineStr">
@@ -22190,7 +22190,7 @@
       </c>
       <c r="B435" s="2" t="inlineStr">
         <is>
-          <t>Cycle MFD Page Backward</t>
+          <t>Strafe Backward</t>
         </is>
       </c>
       <c r="C435" t="inlineStr">
@@ -22243,7 +22243,7 @@
       </c>
       <c r="B436" s="2" t="inlineStr">
         <is>
-          <t>Trigger Down</t>
+          <t>Strafe Down</t>
         </is>
       </c>
       <c r="C436" t="inlineStr">
@@ -22296,7 +22296,7 @@
       </c>
       <c r="B437" s="2" t="inlineStr">
         <is>
-          <t>Cycle MFD Page Forward</t>
+          <t>Strafe Forward</t>
         </is>
       </c>
       <c r="C437" t="inlineStr">
@@ -22349,7 +22349,7 @@
       </c>
       <c r="B438" s="2" t="inlineStr">
         <is>
-          <t>Select Left Head</t>
+          <t>Strafe Left/Right</t>
         </is>
       </c>
       <c r="C438" t="inlineStr">
@@ -22402,7 +22402,7 @@
       </c>
       <c r="B439" s="2" t="inlineStr">
         <is>
-          <t>Select Left Head</t>
+          <t>Strafe Left</t>
         </is>
       </c>
       <c r="C439" t="inlineStr">
@@ -22455,7 +22455,7 @@
       </c>
       <c r="B440" s="2" t="inlineStr">
         <is>
-          <t>Cycle MFD Page Backward</t>
+          <t>Strafe Forward/Backward</t>
         </is>
       </c>
       <c r="C440" t="inlineStr">
@@ -22508,7 +22508,7 @@
       </c>
       <c r="B441" s="2" t="inlineStr">
         <is>
-          <t>Cycle Right Tool</t>
+          <t>Strafe Right</t>
         </is>
       </c>
       <c r="C441" t="inlineStr">
@@ -22561,7 +22561,7 @@
       </c>
       <c r="B442" s="2" t="inlineStr">
         <is>
-          <t>Trigger Up</t>
+          <t>Strafe Up</t>
         </is>
       </c>
       <c r="C442" t="inlineStr">
@@ -22614,7 +22614,7 @@
       </c>
       <c r="B443" s="2" t="inlineStr">
         <is>
-          <t>Trigger Up</t>
+          <t>Strafe Up/Down</t>
         </is>
       </c>
       <c r="C443" t="inlineStr">
@@ -22667,7 +22667,7 @@
       </c>
       <c r="B444" s="2" t="inlineStr">
         <is>
-          <t>Reset Freelook Toggle</t>
+          <t>Reset Freelook</t>
         </is>
       </c>
       <c r="C444" t="inlineStr">
@@ -22720,7 +22720,7 @@
       </c>
       <c r="B445" s="2" t="inlineStr">
         <is>
-          <t>Trigger Up</t>
+          <t>View Up/Down</t>
         </is>
       </c>
       <c r="C445" t="inlineStr">
@@ -22773,7 +22773,7 @@
       </c>
       <c r="B446" s="2" t="inlineStr">
         <is>
-          <t>Trigger Down</t>
+          <t>View Down</t>
         </is>
       </c>
       <c r="C446" t="inlineStr">
@@ -22826,7 +22826,7 @@
       </c>
       <c r="B447" s="2" t="inlineStr">
         <is>
-          <t>Turret Mouse Mode*</t>
+          <t>View Up/Down</t>
         </is>
       </c>
       <c r="C447" t="inlineStr">
@@ -22879,7 +22879,7 @@
       </c>
       <c r="B448" s="2" t="inlineStr">
         <is>
-          <t>Trigger Up</t>
+          <t>View Up</t>
         </is>
       </c>
       <c r="C448" t="inlineStr">
@@ -22932,7 +22932,7 @@
       </c>
       <c r="B449" s="2" t="inlineStr">
         <is>
-          <t>Select Left Head</t>
+          <t>View Left/Right</t>
         </is>
       </c>
       <c r="C449" t="inlineStr">
@@ -22985,7 +22985,7 @@
       </c>
       <c r="B450" s="2" t="inlineStr">
         <is>
-          <t>Select Left Head</t>
+          <t>View Left</t>
         </is>
       </c>
       <c r="C450" t="inlineStr">
@@ -23038,7 +23038,7 @@
       </c>
       <c r="B451" s="2" t="inlineStr">
         <is>
-          <t>Turret Mouse Mode*</t>
+          <t>View Left/Right</t>
         </is>
       </c>
       <c r="C451" t="inlineStr">
@@ -23091,7 +23091,7 @@
       </c>
       <c r="B452" s="2" t="inlineStr">
         <is>
-          <t>Cycle Right Tool</t>
+          <t>View Right</t>
         </is>
       </c>
       <c r="C452" t="inlineStr">
@@ -23226,7 +23226,7 @@
       </c>
       <c r="B455" s="2" t="inlineStr">
         <is>
-          <t>Select Left Head</t>
+          <t>Roll Left</t>
         </is>
       </c>
       <c r="C455" t="inlineStr">
@@ -23279,7 +23279,7 @@
       </c>
       <c r="B456" s="2" t="inlineStr">
         <is>
-          <t>Cycle Right Tool</t>
+          <t>Roll Right</t>
         </is>
       </c>
       <c r="C456" t="inlineStr">

</xml_diff>

<commit_message>
tools: Pin Index N -> Pin N; Pin/Unpin format; manual fixes for chart-mismatched indices
</commit_message>
<xml_diff>
--- a/dev/humanlabel-review.xlsx
+++ b/dev/humanlabel-review.xlsx
@@ -14868,7 +14868,7 @@
       </c>
       <c r="B293" s="2" t="inlineStr">
         <is>
-          <t>Unlock Current Target</t>
+          <t>Pin 1 Lock Toggle</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
@@ -14921,7 +14921,7 @@
       </c>
       <c r="B294" s="2" t="inlineStr">
         <is>
-          <t>Pin Index 2 - Lock / Unlock Pinned Target</t>
+          <t>Pin 2 Lock Toggle</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
@@ -14974,7 +14974,7 @@
       </c>
       <c r="B295" s="2" t="inlineStr">
         <is>
-          <t>Pin Index 3 - Lock / Unlock Pinned Target</t>
+          <t>Pin 3 Lock Toggle</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
@@ -15027,7 +15027,7 @@
       </c>
       <c r="B296" s="2" t="inlineStr">
         <is>
-          <t>Pin/Unpin 2</t>
+          <t>Pin/Unpin 1</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
@@ -15080,7 +15080,7 @@
       </c>
       <c r="B297" s="2" t="inlineStr">
         <is>
-          <t>Pin Index 1 - Pin / Unpin Selected Target</t>
+          <t>Pin/Unpin 1</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
@@ -15133,7 +15133,7 @@
       </c>
       <c r="B298" s="2" t="inlineStr">
         <is>
-          <t>Pin Index 2 - Pin / Unpin Selected Target</t>
+          <t>Pin/Unpin 2</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
@@ -15186,7 +15186,7 @@
       </c>
       <c r="B299" s="2" t="inlineStr">
         <is>
-          <t>Pin Index 2 - Pin / Unpin Selected Target</t>
+          <t>Pin/Unpin 2</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
@@ -15239,7 +15239,7 @@
       </c>
       <c r="B300" s="2" t="inlineStr">
         <is>
-          <t>Pin Index 3 - Pin / Unpin Selected Target</t>
+          <t>Pin/Unpin 3</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
@@ -15292,7 +15292,7 @@
       </c>
       <c r="B301" s="2" t="inlineStr">
         <is>
-          <t>Pin Index 3 - Pin / Unpin Selected Target</t>
+          <t>Pin/Unpin 3</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
@@ -17286,7 +17286,7 @@
       </c>
       <c r="B339" s="2" t="inlineStr">
         <is>
-          <t>Staggered Fire - On / Off Toggle</t>
+          <t>Staggered Fire - On/Off Toggle</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
@@ -18192,7 +18192,7 @@
       </c>
       <c r="B357" s="2" t="inlineStr">
         <is>
-          <t>Turret E.S.P. On / Off Toggle</t>
+          <t>Turret E.S.P. On/Off Toggle</t>
         </is>
       </c>
       <c r="C357" t="inlineStr">

</xml_diff>

<commit_message>
tools: split afterburner vs boost (XML-name driven label)
</commit_message>
<xml_diff>
--- a/dev/humanlabel-review.xlsx
+++ b/dev/humanlabel-review.xlsx
@@ -8131,7 +8131,7 @@
       </c>
       <c r="B160" s="2" t="inlineStr">
         <is>
-          <t>Invoke Docking Toggle</t>
+          <t>Invoke Docking</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
@@ -14921,7 +14921,7 @@
       </c>
       <c r="B294" s="2" t="inlineStr">
         <is>
-          <t>Pin 2 Lock Toggle</t>
+          <t>Unlock Current Target</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
@@ -15080,7 +15080,7 @@
       </c>
       <c r="B297" s="2" t="inlineStr">
         <is>
-          <t>Pin/Unpin 1</t>
+          <t>Pin/Unpin 2</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
@@ -21949,7 +21949,7 @@
       </c>
       <c r="B430" s="2" t="inlineStr">
         <is>
-          <t>After Burner</t>
+          <t>Boost</t>
         </is>
       </c>
       <c r="C430" t="inlineStr">
@@ -23661,7 +23661,7 @@
       <c r="A466" t="inlineStr"/>
       <c r="B466" s="2" t="inlineStr">
         <is>
-          <t>After Burner</t>
+          <t>Boost</t>
         </is>
       </c>
       <c r="C466" t="inlineStr">

</xml_diff>

<commit_message>
tools: eva_ prefix; _long/_hold -> [H] suffix; manual overrides for chart-mismatched indices
</commit_message>
<xml_diff>
--- a/dev/humanlabel-review.xlsx
+++ b/dev/humanlabel-review.xlsx
@@ -1358,7 +1358,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Pin Selected</t>
+          <t>Pin Selected [H]</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1464,7 +1464,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Unpin Selected</t>
+          <t>Unpin Selected [H]</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Select MFD Cast Left</t>
+          <t>Select MFD Cast Left [H]</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2614,7 +2614,7 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Select MFD Cast Right</t>
+          <t>Select MFD Cast Right [H]</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -9506,7 +9506,7 @@
       <c r="A187" t="inlineStr"/>
       <c r="B187" s="2" t="inlineStr">
         <is>
-          <t>Bomb Impact Toggle</t>
+          <t>Bomb Impact Toggle [H]</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
@@ -9820,7 +9820,7 @@
       <c r="A193" t="inlineStr"/>
       <c r="B193" s="2" t="inlineStr">
         <is>
-          <t>Weapon Launch Missile Cinematic</t>
+          <t>Missile Cinematic Camera [H]</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
@@ -11007,7 +11007,7 @@
       </c>
       <c r="B216" s="2" t="inlineStr">
         <is>
-          <t>Master Mode Cycle</t>
+          <t>Master Mode Cycle [H]</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
@@ -11570,7 +11570,7 @@
       </c>
       <c r="B227" s="2" t="inlineStr">
         <is>
-          <t>Forward / Back</t>
+          <t>Throttle Forward / Back</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
@@ -11623,7 +11623,7 @@
       </c>
       <c r="B228" s="2" t="inlineStr">
         <is>
-          <t>Forward / Back Invert</t>
+          <t>Throttle Forward / Back Invert</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
@@ -11729,7 +11729,7 @@
       </c>
       <c r="B230" s="2" t="inlineStr">
         <is>
-          <t>Release Trim</t>
+          <t>Release Trim [H]</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
@@ -11835,7 +11835,7 @@
       </c>
       <c r="B232" s="2" t="inlineStr">
         <is>
-          <t>Set Trim 100%</t>
+          <t>Set Trim 100% [H]</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
@@ -11888,7 +11888,7 @@
       </c>
       <c r="B233" s="2" t="inlineStr">
         <is>
-          <t>Trim - Set To 50%</t>
+          <t>Set Trim 50% [H]</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
@@ -11941,7 +11941,7 @@
       </c>
       <c r="B234" s="2" t="inlineStr">
         <is>
-          <t>Trim - Set To 50%</t>
+          <t>Set Trim 50%</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
@@ -11994,7 +11994,7 @@
       </c>
       <c r="B235" s="2" t="inlineStr">
         <is>
-          <t>Trim - Set</t>
+          <t>Set Trim</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
@@ -14607,7 +14607,7 @@
       </c>
       <c r="B288" s="2" t="inlineStr">
         <is>
-          <t>Auto Targeting - On/Off Toggle</t>
+          <t>Power On/Off Toggle [H]</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
@@ -14921,7 +14921,7 @@
       </c>
       <c r="B294" s="2" t="inlineStr">
         <is>
-          <t>Unlock Current Target</t>
+          <t>Pin 2 Lock Toggle</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
@@ -15080,7 +15080,7 @@
       </c>
       <c r="B297" s="2" t="inlineStr">
         <is>
-          <t>Pin/Unpin 2</t>
+          <t>Pin/Unpin 1 [H]</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
@@ -15186,7 +15186,7 @@
       </c>
       <c r="B299" s="2" t="inlineStr">
         <is>
-          <t>Pin/Unpin 2</t>
+          <t>Pin/Unpin 2 [H]</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
@@ -15292,7 +15292,7 @@
       </c>
       <c r="B301" s="2" t="inlineStr">
         <is>
-          <t>Pin/Unpin 3</t>
+          <t>Pin/Unpin 3 [H]</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
@@ -15924,7 +15924,7 @@
       <c r="A313" t="inlineStr"/>
       <c r="B313" s="2" t="inlineStr">
         <is>
-          <t>ADS</t>
+          <t>ADS Zoom Toggle [H]</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
@@ -15965,7 +15965,7 @@
       <c r="A314" t="inlineStr"/>
       <c r="B314" s="2" t="inlineStr">
         <is>
-          <t>ADS Stable Max Zoom</t>
+          <t>ADS Stable Max Zoom [H]</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -20509,7 +20509,7 @@
       </c>
       <c r="B402" s="2" t="inlineStr">
         <is>
-          <t>Cycle Page - Backwards</t>
+          <t>Cycle MFD Page Backward [H]</t>
         </is>
       </c>
       <c r="C402" t="inlineStr">
@@ -20615,7 +20615,7 @@
       </c>
       <c r="B404" s="2" t="inlineStr">
         <is>
-          <t>Cycle Page - Forwards</t>
+          <t>Cycle MFD Page Forward [H]</t>
         </is>
       </c>
       <c r="C404" t="inlineStr">
@@ -20721,7 +20721,7 @@
       </c>
       <c r="B406" s="2" t="inlineStr">
         <is>
-          <t>Movement - Down</t>
+          <t>Select MFD Down [H]</t>
         </is>
       </c>
       <c r="C406" t="inlineStr">
@@ -20774,7 +20774,7 @@
       </c>
       <c r="B407" s="2" t="inlineStr">
         <is>
-          <t>Select MFD Left</t>
+          <t>Select MFD Left [H]</t>
         </is>
       </c>
       <c r="C407" t="inlineStr">
@@ -20827,7 +20827,7 @@
       </c>
       <c r="B408" s="2" t="inlineStr">
         <is>
-          <t>Select MFD Right</t>
+          <t>Select MFD Right [H]</t>
         </is>
       </c>
       <c r="C408" t="inlineStr">
@@ -20880,7 +20880,7 @@
       </c>
       <c r="B409" s="2" t="inlineStr">
         <is>
-          <t>Movement - Up</t>
+          <t>Select MFD Up [H]</t>
         </is>
       </c>
       <c r="C409" t="inlineStr">
@@ -21357,7 +21357,7 @@
       </c>
       <c r="B418" s="2" t="inlineStr">
         <is>
-          <t>Select - MFD 1</t>
+          <t>Select - MFD 1 [H]</t>
         </is>
       </c>
       <c r="C418" t="inlineStr">
@@ -21410,7 +21410,7 @@
       </c>
       <c r="B419" s="2" t="inlineStr">
         <is>
-          <t>Select - MFD 2</t>
+          <t>Select - MFD 2 [H]</t>
         </is>
       </c>
       <c r="C419" t="inlineStr">
@@ -21463,7 +21463,7 @@
       </c>
       <c r="B420" s="2" t="inlineStr">
         <is>
-          <t>Select - MFD 3</t>
+          <t>Select - MFD 3 [H]</t>
         </is>
       </c>
       <c r="C420" t="inlineStr">
@@ -21516,7 +21516,7 @@
       </c>
       <c r="B421" s="2" t="inlineStr">
         <is>
-          <t>Select - MFD 4</t>
+          <t>Select - MFD 4 [H]</t>
         </is>
       </c>
       <c r="C421" t="inlineStr">
@@ -21569,7 +21569,7 @@
       </c>
       <c r="B422" s="2" t="inlineStr">
         <is>
-          <t>Select - MFD 5</t>
+          <t>Select - MFD 5 [H]</t>
         </is>
       </c>
       <c r="C422" t="inlineStr">
@@ -21622,7 +21622,7 @@
       </c>
       <c r="B423" s="2" t="inlineStr">
         <is>
-          <t>Select - MFD 6</t>
+          <t>Select - MFD 6 [H]</t>
         </is>
       </c>
       <c r="C423" t="inlineStr">
@@ -21675,7 +21675,7 @@
       </c>
       <c r="B424" s="2" t="inlineStr">
         <is>
-          <t>Select - MFD 7</t>
+          <t>Select - MFD 7 [H]</t>
         </is>
       </c>
       <c r="C424" t="inlineStr">
@@ -21728,7 +21728,7 @@
       </c>
       <c r="B425" s="2" t="inlineStr">
         <is>
-          <t>Select - MFD 8</t>
+          <t>Select - MFD 8 [H]</t>
         </is>
       </c>
       <c r="C425" t="inlineStr">
@@ -21949,7 +21949,7 @@
       </c>
       <c r="B430" s="2" t="inlineStr">
         <is>
-          <t>Boost</t>
+          <t>EVA Boost</t>
         </is>
       </c>
       <c r="C430" t="inlineStr">
@@ -21990,7 +21990,7 @@
       </c>
       <c r="B431" s="2" t="inlineStr">
         <is>
-          <t>Brake</t>
+          <t>EVA Brake</t>
         </is>
       </c>
       <c r="C431" t="inlineStr">
@@ -22031,7 +22031,7 @@
       </c>
       <c r="B432" s="2" t="inlineStr">
         <is>
-          <t>Roll Left/Right</t>
+          <t>EVA Roll Left/Right</t>
         </is>
       </c>
       <c r="C432" t="inlineStr">
@@ -22084,7 +22084,7 @@
       </c>
       <c r="B433" s="2" t="inlineStr">
         <is>
-          <t>Roll Left</t>
+          <t>EVA Roll Left</t>
         </is>
       </c>
       <c r="C433" t="inlineStr">
@@ -22137,7 +22137,7 @@
       </c>
       <c r="B434" s="2" t="inlineStr">
         <is>
-          <t>Roll Right</t>
+          <t>EVA Roll Right</t>
         </is>
       </c>
       <c r="C434" t="inlineStr">
@@ -22190,7 +22190,7 @@
       </c>
       <c r="B435" s="2" t="inlineStr">
         <is>
-          <t>Strafe Backward</t>
+          <t>EVA Strafe Backward</t>
         </is>
       </c>
       <c r="C435" t="inlineStr">
@@ -22243,7 +22243,7 @@
       </c>
       <c r="B436" s="2" t="inlineStr">
         <is>
-          <t>Strafe Down</t>
+          <t>EVA Strafe Down</t>
         </is>
       </c>
       <c r="C436" t="inlineStr">
@@ -22296,7 +22296,7 @@
       </c>
       <c r="B437" s="2" t="inlineStr">
         <is>
-          <t>Strafe Forward</t>
+          <t>EVA Strafe Forward</t>
         </is>
       </c>
       <c r="C437" t="inlineStr">
@@ -22349,7 +22349,7 @@
       </c>
       <c r="B438" s="2" t="inlineStr">
         <is>
-          <t>Strafe Left/Right</t>
+          <t>EVA Strafe Left/Right</t>
         </is>
       </c>
       <c r="C438" t="inlineStr">
@@ -22402,7 +22402,7 @@
       </c>
       <c r="B439" s="2" t="inlineStr">
         <is>
-          <t>Strafe Left</t>
+          <t>EVA Strafe Left</t>
         </is>
       </c>
       <c r="C439" t="inlineStr">
@@ -22455,7 +22455,7 @@
       </c>
       <c r="B440" s="2" t="inlineStr">
         <is>
-          <t>Strafe Forward/Backward</t>
+          <t>EVA Strafe Forward/Backward</t>
         </is>
       </c>
       <c r="C440" t="inlineStr">
@@ -22508,7 +22508,7 @@
       </c>
       <c r="B441" s="2" t="inlineStr">
         <is>
-          <t>Strafe Right</t>
+          <t>EVA Strafe Right</t>
         </is>
       </c>
       <c r="C441" t="inlineStr">
@@ -22561,7 +22561,7 @@
       </c>
       <c r="B442" s="2" t="inlineStr">
         <is>
-          <t>Strafe Up</t>
+          <t>EVA Strafe Up</t>
         </is>
       </c>
       <c r="C442" t="inlineStr">
@@ -22614,7 +22614,7 @@
       </c>
       <c r="B443" s="2" t="inlineStr">
         <is>
-          <t>Strafe Up/Down</t>
+          <t>EVA Strafe Up/Down</t>
         </is>
       </c>
       <c r="C443" t="inlineStr">
@@ -22667,7 +22667,7 @@
       </c>
       <c r="B444" s="2" t="inlineStr">
         <is>
-          <t>Reset Freelook</t>
+          <t>EVA Freelook</t>
         </is>
       </c>
       <c r="C444" t="inlineStr">
@@ -22720,7 +22720,7 @@
       </c>
       <c r="B445" s="2" t="inlineStr">
         <is>
-          <t>View Up/Down</t>
+          <t>EVA View Up/Down</t>
         </is>
       </c>
       <c r="C445" t="inlineStr">
@@ -22773,7 +22773,7 @@
       </c>
       <c r="B446" s="2" t="inlineStr">
         <is>
-          <t>View Down</t>
+          <t>EVA View Down</t>
         </is>
       </c>
       <c r="C446" t="inlineStr">
@@ -22826,7 +22826,7 @@
       </c>
       <c r="B447" s="2" t="inlineStr">
         <is>
-          <t>View Up/Down</t>
+          <t>EVA View Up/Down</t>
         </is>
       </c>
       <c r="C447" t="inlineStr">
@@ -22879,7 +22879,7 @@
       </c>
       <c r="B448" s="2" t="inlineStr">
         <is>
-          <t>View Up</t>
+          <t>EVA View Up</t>
         </is>
       </c>
       <c r="C448" t="inlineStr">
@@ -22932,7 +22932,7 @@
       </c>
       <c r="B449" s="2" t="inlineStr">
         <is>
-          <t>View Left/Right</t>
+          <t>EVA View Left/Right</t>
         </is>
       </c>
       <c r="C449" t="inlineStr">
@@ -22985,7 +22985,7 @@
       </c>
       <c r="B450" s="2" t="inlineStr">
         <is>
-          <t>View Left</t>
+          <t>EVA View Left</t>
         </is>
       </c>
       <c r="C450" t="inlineStr">
@@ -23038,7 +23038,7 @@
       </c>
       <c r="B451" s="2" t="inlineStr">
         <is>
-          <t>View Left/Right</t>
+          <t>EVA View Left/Right</t>
         </is>
       </c>
       <c r="C451" t="inlineStr">
@@ -23091,7 +23091,7 @@
       </c>
       <c r="B452" s="2" t="inlineStr">
         <is>
-          <t>View Right</t>
+          <t>EVA View Right</t>
         </is>
       </c>
       <c r="C452" t="inlineStr">

</xml_diff>

<commit_message>
tools: move [H] from suffix to prefix on _long/_hold actions
</commit_message>
<xml_diff>
--- a/dev/humanlabel-review.xlsx
+++ b/dev/humanlabel-review.xlsx
@@ -1358,7 +1358,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Pin Selected [H]</t>
+          <t>[H] Pin Selected</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1464,7 +1464,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Unpin Selected [H]</t>
+          <t>[H] Unpin Selected</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Select MFD Cast Left [H]</t>
+          <t>[H] Select MFD Cast Left</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2614,7 +2614,7 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Select MFD Cast Right [H]</t>
+          <t>[H] Select MFD Cast Right</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -9506,7 +9506,7 @@
       <c r="A187" t="inlineStr"/>
       <c r="B187" s="2" t="inlineStr">
         <is>
-          <t>Bomb Impact Toggle [H]</t>
+          <t>[H] Bomb Impact Toggle</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
@@ -9820,7 +9820,7 @@
       <c r="A193" t="inlineStr"/>
       <c r="B193" s="2" t="inlineStr">
         <is>
-          <t>Missile Cinematic Camera [H]</t>
+          <t>[H] Missile Cinematic Camera</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
@@ -11007,7 +11007,7 @@
       </c>
       <c r="B216" s="2" t="inlineStr">
         <is>
-          <t>Master Mode Cycle [H]</t>
+          <t>[H] Master Mode Cycle</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
@@ -11729,7 +11729,7 @@
       </c>
       <c r="B230" s="2" t="inlineStr">
         <is>
-          <t>Release Trim [H]</t>
+          <t>[H] Release Trim</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
@@ -11835,7 +11835,7 @@
       </c>
       <c r="B232" s="2" t="inlineStr">
         <is>
-          <t>Set Trim 100% [H]</t>
+          <t>[H] Set Trim 100%</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
@@ -11888,7 +11888,7 @@
       </c>
       <c r="B233" s="2" t="inlineStr">
         <is>
-          <t>Set Trim 50% [H]</t>
+          <t>[H] Set Trim 50%</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
@@ -14607,7 +14607,7 @@
       </c>
       <c r="B288" s="2" t="inlineStr">
         <is>
-          <t>Power On/Off Toggle [H]</t>
+          <t>[H] Power On/Off Toggle</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
@@ -15080,7 +15080,7 @@
       </c>
       <c r="B297" s="2" t="inlineStr">
         <is>
-          <t>Pin/Unpin 1 [H]</t>
+          <t>[H] Pin/Unpin 1</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
@@ -15186,7 +15186,7 @@
       </c>
       <c r="B299" s="2" t="inlineStr">
         <is>
-          <t>Pin/Unpin 2 [H]</t>
+          <t>[H] Pin/Unpin 2</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
@@ -15292,7 +15292,7 @@
       </c>
       <c r="B301" s="2" t="inlineStr">
         <is>
-          <t>Pin/Unpin 3 [H]</t>
+          <t>[H] Pin/Unpin 3</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
@@ -15924,7 +15924,7 @@
       <c r="A313" t="inlineStr"/>
       <c r="B313" s="2" t="inlineStr">
         <is>
-          <t>ADS Zoom Toggle [H]</t>
+          <t>[H] ADS Zoom Toggle</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
@@ -15965,7 +15965,7 @@
       <c r="A314" t="inlineStr"/>
       <c r="B314" s="2" t="inlineStr">
         <is>
-          <t>ADS Stable Max Zoom [H]</t>
+          <t>[H] ADS Stable Max Zoom</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -20509,7 +20509,7 @@
       </c>
       <c r="B402" s="2" t="inlineStr">
         <is>
-          <t>Cycle MFD Page Backward [H]</t>
+          <t>[H] Cycle MFD Page Backward</t>
         </is>
       </c>
       <c r="C402" t="inlineStr">
@@ -20615,7 +20615,7 @@
       </c>
       <c r="B404" s="2" t="inlineStr">
         <is>
-          <t>Cycle MFD Page Forward [H]</t>
+          <t>[H] Cycle MFD Page Forward</t>
         </is>
       </c>
       <c r="C404" t="inlineStr">
@@ -20721,7 +20721,7 @@
       </c>
       <c r="B406" s="2" t="inlineStr">
         <is>
-          <t>Select MFD Down [H]</t>
+          <t>[H] Select MFD Down</t>
         </is>
       </c>
       <c r="C406" t="inlineStr">
@@ -20774,7 +20774,7 @@
       </c>
       <c r="B407" s="2" t="inlineStr">
         <is>
-          <t>Select MFD Left [H]</t>
+          <t>[H] Select MFD Left</t>
         </is>
       </c>
       <c r="C407" t="inlineStr">
@@ -20827,7 +20827,7 @@
       </c>
       <c r="B408" s="2" t="inlineStr">
         <is>
-          <t>Select MFD Right [H]</t>
+          <t>[H] Select MFD Right</t>
         </is>
       </c>
       <c r="C408" t="inlineStr">
@@ -20880,7 +20880,7 @@
       </c>
       <c r="B409" s="2" t="inlineStr">
         <is>
-          <t>Select MFD Up [H]</t>
+          <t>[H] Select MFD Up</t>
         </is>
       </c>
       <c r="C409" t="inlineStr">
@@ -21357,7 +21357,7 @@
       </c>
       <c r="B418" s="2" t="inlineStr">
         <is>
-          <t>Select - MFD 1 [H]</t>
+          <t>[H] Select - MFD 1</t>
         </is>
       </c>
       <c r="C418" t="inlineStr">
@@ -21410,7 +21410,7 @@
       </c>
       <c r="B419" s="2" t="inlineStr">
         <is>
-          <t>Select - MFD 2 [H]</t>
+          <t>[H] Select - MFD 2</t>
         </is>
       </c>
       <c r="C419" t="inlineStr">
@@ -21463,7 +21463,7 @@
       </c>
       <c r="B420" s="2" t="inlineStr">
         <is>
-          <t>Select - MFD 3 [H]</t>
+          <t>[H] Select - MFD 3</t>
         </is>
       </c>
       <c r="C420" t="inlineStr">
@@ -21516,7 +21516,7 @@
       </c>
       <c r="B421" s="2" t="inlineStr">
         <is>
-          <t>Select - MFD 4 [H]</t>
+          <t>[H] Select - MFD 4</t>
         </is>
       </c>
       <c r="C421" t="inlineStr">
@@ -21569,7 +21569,7 @@
       </c>
       <c r="B422" s="2" t="inlineStr">
         <is>
-          <t>Select - MFD 5 [H]</t>
+          <t>[H] Select - MFD 5</t>
         </is>
       </c>
       <c r="C422" t="inlineStr">
@@ -21622,7 +21622,7 @@
       </c>
       <c r="B423" s="2" t="inlineStr">
         <is>
-          <t>Select - MFD 6 [H]</t>
+          <t>[H] Select - MFD 6</t>
         </is>
       </c>
       <c r="C423" t="inlineStr">
@@ -21675,7 +21675,7 @@
       </c>
       <c r="B424" s="2" t="inlineStr">
         <is>
-          <t>Select - MFD 7 [H]</t>
+          <t>[H] Select - MFD 7</t>
         </is>
       </c>
       <c r="C424" t="inlineStr">
@@ -21728,7 +21728,7 @@
       </c>
       <c r="B425" s="2" t="inlineStr">
         <is>
-          <t>Select - MFD 8 [H]</t>
+          <t>[H] Select - MFD 8</t>
         </is>
       </c>
       <c r="C425" t="inlineStr">

</xml_diff>

<commit_message>
tools: Next/Prev. as suffix + Cycle Lock override + Weapon Presets singularize
</commit_message>
<xml_diff>
--- a/dev/humanlabel-review.xlsx
+++ b/dev/humanlabel-review.xlsx
@@ -664,7 +664,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Prev. Operator Mode</t>
+          <t>Operator Mode Prev.</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -717,7 +717,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Next Operator Mode</t>
+          <t>Operator Mode Next</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1517,7 +1517,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Attackers Target Backward</t>
+          <t>Attacker Target Back</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1570,7 +1570,7 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Target Attacker Forward</t>
+          <t>Attacker Target Forward</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1623,7 +1623,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Target Attacker Closest</t>
+          <t>Attacker Target Closest</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1676,7 +1676,7 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Friendly Target Backward</t>
+          <t>Friendly Target Back</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1835,7 +1835,7 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Door Lock Cycle</t>
+          <t>In-View Target Forward</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1941,7 +1941,7 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Sub Target Reset Main</t>
+          <t>Sub Target Target - Reset to Main Target</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -2088,7 +2088,7 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Next Weapon Preset</t>
+          <t>Weapon Preset Next</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -2141,7 +2141,7 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Next Weapon Preset (Overflow)</t>
+          <t>Weapon Preset Next (Overflow)</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -2194,7 +2194,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Next Remote Turret*</t>
+          <t>Remote Turret Next*</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2247,7 +2247,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Previous Remote Turret*</t>
+          <t>Remote Turret Prev.*</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -3104,7 +3104,7 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Fire Right Tool</t>
+          <t>Tool Secondary Fire</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -3643,7 +3643,7 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Next Weapon Presett</t>
+          <t>Weapon Next</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -3798,7 +3798,7 @@
       <c r="A67" t="inlineStr"/>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>Prev. Item</t>
+          <t>Item Prev.</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -3851,7 +3851,7 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>Prev. Weapon Preset</t>
+          <t>Weapon Prev.</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -3945,7 +3945,7 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>Camera (3rd Person)</t>
+          <t>Third Person</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -6691,7 +6691,7 @@
       </c>
       <c r="B132" s="2" t="inlineStr">
         <is>
-          <t>Enable / Disable Head Tracking for 3rd Person Camera</t>
+          <t>Camera (3rd Person)</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
@@ -7499,7 +7499,7 @@
       </c>
       <c r="B148" s="2" t="inlineStr">
         <is>
-          <t>Shield Cap Increase</t>
+          <t>Shield Cap Inc.</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
@@ -9559,7 +9559,7 @@
       </c>
       <c r="B188" s="2" t="inlineStr">
         <is>
-          <t>Missile Type Previous</t>
+          <t>Missile Type Prev.</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
@@ -14293,7 +14293,7 @@
       <c r="A282" t="inlineStr"/>
       <c r="B282" s="2" t="inlineStr">
         <is>
-          <t>Salvage Fire Right Toggle</t>
+          <t>Fire Right Tool</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
@@ -15398,7 +15398,7 @@
       </c>
       <c r="B303" s="2" t="inlineStr">
         <is>
-          <t>All Target Backward</t>
+          <t>All Target Back</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
@@ -15557,7 +15557,7 @@
       </c>
       <c r="B306" s="2" t="inlineStr">
         <is>
-          <t>Hostile Target Backward</t>
+          <t>Hostile Target Back</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
@@ -15716,7 +15716,7 @@
       </c>
       <c r="B309" s="2" t="inlineStr">
         <is>
-          <t>Target Under Reticle</t>
+          <t>In-View Target Under Reticle</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
@@ -15769,7 +15769,7 @@
       </c>
       <c r="B310" s="2" t="inlineStr">
         <is>
-          <t>Sub Target Backward</t>
+          <t>Sub Target Target - Back</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
@@ -15822,7 +15822,7 @@
       </c>
       <c r="B311" s="2" t="inlineStr">
         <is>
-          <t>Sub Target Forward</t>
+          <t>Sub Target Target - Forward</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
@@ -15875,7 +15875,7 @@
       </c>
       <c r="B312" s="2" t="inlineStr">
         <is>
-          <t>Lock Target Under Reticle</t>
+          <t>Target Under Reticle</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
@@ -16597,7 +16597,7 @@
       </c>
       <c r="B326" s="2" t="inlineStr">
         <is>
-          <t>Weapon Preset - Fire</t>
+          <t>Weapon Preset Prev.</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
@@ -16756,7 +16756,7 @@
       </c>
       <c r="B329" s="2" t="inlineStr">
         <is>
-          <t>Weapon Presets - Fire Guns Group 2</t>
+          <t>Weapon Preset Fire Guns Group 2</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
@@ -16809,7 +16809,7 @@
       </c>
       <c r="B330" s="2" t="inlineStr">
         <is>
-          <t>Weapon Presets - Fire Guns Group 3</t>
+          <t>Weapon Preset Fire Guns Group 3</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
@@ -16862,7 +16862,7 @@
       </c>
       <c r="B331" s="2" t="inlineStr">
         <is>
-          <t>Weapon Presets - Fire Guns Group 4</t>
+          <t>Weapon Preset Fire Guns Group 4</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
@@ -16915,7 +16915,7 @@
       </c>
       <c r="B332" s="2" t="inlineStr">
         <is>
-          <t>Weapon Presets - Set Guns Group 1</t>
+          <t>Weapon Preset Set Guns Group 1</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
@@ -16968,7 +16968,7 @@
       </c>
       <c r="B333" s="2" t="inlineStr">
         <is>
-          <t>Weapon Presets - Set Guns Group 2</t>
+          <t>Weapon Preset Set Guns Group 2</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
@@ -17021,7 +17021,7 @@
       </c>
       <c r="B334" s="2" t="inlineStr">
         <is>
-          <t>Weapon Presets - Prev.</t>
+          <t>Weapon Preset Prev.</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
@@ -17074,7 +17074,7 @@
       </c>
       <c r="B335" s="2" t="inlineStr">
         <is>
-          <t>Prev. Weapon Preset (Overflow)</t>
+          <t>Weapon Preset Prev. (Overflow)</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
@@ -17127,7 +17127,7 @@
       </c>
       <c r="B336" s="2" t="inlineStr">
         <is>
-          <t>Weapon Presets - Set QIDs</t>
+          <t>Weapon Preset Set QIDs</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
@@ -17180,7 +17180,7 @@
       </c>
       <c r="B337" s="2" t="inlineStr">
         <is>
-          <t>Weapon Presets - Set Quantum Jammers (short range)</t>
+          <t>Weapon Preset Set Quantum Jammers (short range)</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
@@ -17233,7 +17233,7 @@
       </c>
       <c r="B338" s="2" t="inlineStr">
         <is>
-          <t>Weapon Presets - Set Quantum Snares / Pulse (long range)</t>
+          <t>Weapon Preset Set Quantum Snares / Pulse (long range)</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
@@ -23402,7 +23402,7 @@
       <c r="A459" t="inlineStr"/>
       <c r="B459" s="2" t="inlineStr">
         <is>
-          <t>Next Item</t>
+          <t>Item Next</t>
         </is>
       </c>
       <c r="C459" t="inlineStr">

</xml_diff>

<commit_message>
humanlabel: regenerate proposals for SC 4.8.0 LIVE chart corpus
First-pass run after all 5 sticks adopted the Chart Authoring
Conventions. 467 joystick-bound actions matched across 1047
candidate phrases from the refreshed SVGs:

  - 48 high confidence
  - 410 medium
  - 9 low
  - Sources: 392 chart / 66 csv_displayname / 9 xml_fallback

CSV pulled fresh from Monitarr alongside.

humanlabel-review.xlsx ready for mobile review at
https://github.com/SubliminalsTV/Subs-Curated-Bindings/raw/main/tools/humanlabel-review.xlsx
</commit_message>
<xml_diff>
--- a/dev/humanlabel-review.xlsx
+++ b/dev/humanlabel-review.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="HumanLabel Review" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HumanLabel Review" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'HumanLabel Review'!$A$1:$K$468</definedName>

</xml_diff>